<commit_message>
Add initial Excel input file for EmpresaX with Kaizen data
</commit_message>
<xml_diff>
--- a/Inputs_EmpresaX.xlsx
+++ b/Inputs_EmpresaX.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kaizen\Documents\tese\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{358D41FB-D1BC-42A1-91AE-CA373AD38640}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C72EABB-EEF4-4113-AF00-641176C2A83A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -757,8 +757,26 @@
 </comments>
 </file>
 
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={C7364A66-A497-423F-B38F-AF51BEC19DB7}</author>
+  </authors>
+  <commentList>
+    <comment ref="J78" authorId="0" shapeId="0" xr:uid="{C7364A66-A497-423F-B38F-AF51BEC19DB7}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    900</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2146" uniqueCount="528">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2150" uniqueCount="533">
   <si>
     <t>ESTRUTURA FÍSICA DO SISTEMA PRODUTIVO</t>
   </si>
@@ -2342,17 +2360,33 @@
   </si>
   <si>
     <t>DC102600</t>
+  </si>
+  <si>
+    <t>Line</t>
+  </si>
+  <si>
+    <t>Total Occupied Hours</t>
+  </si>
+  <si>
+    <t>Total Available Hours</t>
+  </si>
+  <si>
+    <t>L1</t>
+  </si>
+  <si>
+    <t>L2</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General\ &quot;min&quot;"/>
     <numFmt numFmtId="165" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    <numFmt numFmtId="166" formatCode="0.0"/>
   </numFmts>
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2488,8 +2522,28 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="0"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2539,8 +2593,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF002060"/>
+        <bgColor theme="4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -2654,11 +2714,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="hair">
+        <color indexed="64"/>
+      </left>
+      <right style="hair">
+        <color indexed="64"/>
+      </right>
+      <top style="hair">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="69">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2825,16 +2900,16 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2852,11 +2927,33 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="21" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="20">
+  <dxfs count="21">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -3588,27 +3685,33 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Raquel Duque" id="{DAA1B03B-E46D-4B86-913A-0A7B4214C9B3}" userId="S::rduque@kaizen.com::276b5b66-a20e-4e3a-b701-a469ee4d4468" providerId="AD"/>
+</personList>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{A2E0425D-8D3D-4317-A507-ADC777C31517}" name="Table4" displayName="Table4" ref="A4:Q192" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18" tableBorderDxfId="17">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{A2E0425D-8D3D-4317-A507-ADC777C31517}" name="Table4" displayName="Table4" ref="A4:Q192" totalsRowShown="0" headerRowDxfId="20" dataDxfId="19" tableBorderDxfId="18">
   <autoFilter ref="A4:Q192" xr:uid="{A2E0425D-8D3D-4317-A507-ADC777C31517}"/>
   <tableColumns count="17">
-    <tableColumn id="1" xr3:uid="{26D481BD-1A66-4F75-A5DB-835BDEAD35EC}" name="ref_id" dataDxfId="16"/>
-    <tableColumn id="2" xr3:uid="{AF3D888D-29CC-4818-9F37-35E1C095FEBC}" name="nome" dataDxfId="15"/>
-    <tableColumn id="21" xr3:uid="{A36D18E5-0E2F-48D2-A9EA-1667409CF7FA}" name="Unid_caixa" dataDxfId="14"/>
-    <tableColumn id="19" xr3:uid="{901BF69A-B9CB-436F-8A73-E52E627A4C44}" name="nao_produzir_segunda" dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{73E06642-D2DC-4B3F-B7AE-6A99CF0B73CD}" name="família" dataDxfId="12"/>
-    <tableColumn id="4" xr3:uid="{47F7E5B0-45A6-4E01-8304-DD4D19A9E24E}" name="ativa" dataDxfId="11"/>
-    <tableColumn id="10" xr3:uid="{E576D14B-BDA0-4CA6-B2F4-097D5C1CE99B}" name="pode_L1" dataDxfId="10"/>
-    <tableColumn id="11" xr3:uid="{B29DBEC4-DD50-4914-98AC-30F025559FDC}" name="tempo_L1_prod_min (cadência de L1)" dataDxfId="9"/>
-    <tableColumn id="12" xr3:uid="{14DD02B2-C00E-494B-A8F3-3FFAE31BC4FB}" name="operadores_nec_L1_acab" dataDxfId="8"/>
-    <tableColumn id="13" xr3:uid="{89492EE9-DE84-43EE-B12E-2605FE3EAD79}" name="operadores_nec_L1_prod" dataDxfId="7"/>
-    <tableColumn id="14" xr3:uid="{780BF028-7B4E-42E1-B807-EDB2FB22CEE7}" name="pode_L2" dataDxfId="6"/>
-    <tableColumn id="15" xr3:uid="{FD12F15B-F3BE-48A4-B186-794E71F468D8}" name="tempo_L2_prod_min (cadência de L2)" dataDxfId="5"/>
-    <tableColumn id="16" xr3:uid="{2B695F9C-3774-41DD-8FE4-AF094E98B022}" name="tempo_L2_acab_min (cadência de L2)" dataDxfId="4"/>
-    <tableColumn id="20" xr3:uid="{46C45284-5F2B-442A-A3EB-D66468126784}" name="operadores_nec_L2_acab" dataDxfId="3"/>
-    <tableColumn id="17" xr3:uid="{1453032D-3307-46D2-BB7E-3D55B4D2E43D}" name="operadores_nec_L2_prod" dataDxfId="2"/>
-    <tableColumn id="5" xr3:uid="{5009F860-773A-42AE-9780-72CCCE321658}" name="kg" dataDxfId="1"/>
-    <tableColumn id="18" xr3:uid="{3939DDEA-30DE-43D1-B600-33ECEC5CD680}" name="euros" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{26D481BD-1A66-4F75-A5DB-835BDEAD35EC}" name="ref_id" dataDxfId="17"/>
+    <tableColumn id="2" xr3:uid="{AF3D888D-29CC-4818-9F37-35E1C095FEBC}" name="nome" dataDxfId="16"/>
+    <tableColumn id="21" xr3:uid="{A36D18E5-0E2F-48D2-A9EA-1667409CF7FA}" name="Unid_caixa" dataDxfId="15"/>
+    <tableColumn id="19" xr3:uid="{901BF69A-B9CB-436F-8A73-E52E627A4C44}" name="nao_produzir_segunda" dataDxfId="14"/>
+    <tableColumn id="3" xr3:uid="{73E06642-D2DC-4B3F-B7AE-6A99CF0B73CD}" name="família" dataDxfId="13"/>
+    <tableColumn id="4" xr3:uid="{47F7E5B0-45A6-4E01-8304-DD4D19A9E24E}" name="ativa" dataDxfId="12"/>
+    <tableColumn id="10" xr3:uid="{E576D14B-BDA0-4CA6-B2F4-097D5C1CE99B}" name="pode_L1" dataDxfId="11"/>
+    <tableColumn id="11" xr3:uid="{B29DBEC4-DD50-4914-98AC-30F025559FDC}" name="tempo_L1_prod_min (cadência de L1)" dataDxfId="10"/>
+    <tableColumn id="12" xr3:uid="{14DD02B2-C00E-494B-A8F3-3FFAE31BC4FB}" name="operadores_nec_L1_acab" dataDxfId="9"/>
+    <tableColumn id="13" xr3:uid="{89492EE9-DE84-43EE-B12E-2605FE3EAD79}" name="operadores_nec_L1_prod" dataDxfId="8"/>
+    <tableColumn id="14" xr3:uid="{780BF028-7B4E-42E1-B807-EDB2FB22CEE7}" name="pode_L2" dataDxfId="7"/>
+    <tableColumn id="15" xr3:uid="{FD12F15B-F3BE-48A4-B186-794E71F468D8}" name="tempo_L2_prod_min (cadência de L2)" dataDxfId="6"/>
+    <tableColumn id="16" xr3:uid="{2B695F9C-3774-41DD-8FE4-AF094E98B022}" name="tempo_L2_acab_min (cadência de L2)" dataDxfId="5"/>
+    <tableColumn id="20" xr3:uid="{46C45284-5F2B-442A-A3EB-D66468126784}" name="operadores_nec_L2_acab" dataDxfId="4"/>
+    <tableColumn id="17" xr3:uid="{1453032D-3307-46D2-BB7E-3D55B4D2E43D}" name="operadores_nec_L2_prod" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{5009F860-773A-42AE-9780-72CCCE321658}" name="kg" dataDxfId="2"/>
+    <tableColumn id="18" xr3:uid="{3939DDEA-30DE-43D1-B600-33ECEC5CD680}" name="euros" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3897,6 +4000,14 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="J78" dT="2026-05-21T13:53:57.62" personId="{DAA1B03B-E46D-4B86-913A-0A7B4214C9B3}" id="{C7364A66-A497-423F-B38F-AF51BEC19DB7}">
+    <text>900</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
   <wetp:taskpane dockstate="right" visibility="0" width="525" row="9">
@@ -3983,7 +4094,7 @@
       <c r="C5" s="3"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A6" s="62" t="s">
+      <c r="A6" s="58" t="s">
         <v>5</v>
       </c>
       <c r="B6" s="59"/>
@@ -4020,7 +4131,7 @@
       <c r="C9" s="3"/>
     </row>
     <row r="11" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="62" t="s">
+      <c r="A11" s="58" t="s">
         <v>7</v>
       </c>
       <c r="B11" s="59"/>
@@ -4048,7 +4159,7 @@
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A15" s="62" t="s">
+      <c r="A15" s="58" t="s">
         <v>9</v>
       </c>
       <c r="B15" s="59"/>
@@ -4134,7 +4245,7 @@
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A24" s="62" t="s">
+      <c r="A24" s="58" t="s">
         <v>19</v>
       </c>
       <c r="B24" s="59"/>
@@ -4218,7 +4329,7 @@
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A33" s="62" t="s">
+      <c r="A33" s="58" t="s">
         <v>21</v>
       </c>
       <c r="B33" s="59"/>
@@ -4247,64 +4358,59 @@
       <c r="A39" s="65" t="s">
         <v>42</v>
       </c>
-      <c r="B39" s="61"/>
-      <c r="C39" s="61"/>
+      <c r="B39" s="62"/>
+      <c r="C39" s="62"/>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A40" s="64" t="s">
         <v>24</v>
       </c>
-      <c r="B40" s="61"/>
-      <c r="C40" s="61"/>
+      <c r="B40" s="62"/>
+      <c r="C40" s="62"/>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A41" s="64"/>
-      <c r="B41" s="61"/>
-      <c r="C41" s="61"/>
+      <c r="B41" s="62"/>
+      <c r="C41" s="62"/>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A42" s="63" t="s">
         <v>25</v>
       </c>
-      <c r="B42" s="61"/>
-      <c r="C42" s="61"/>
+      <c r="B42" s="62"/>
+      <c r="C42" s="62"/>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A43" s="60" t="s">
+      <c r="A43" s="61" t="s">
         <v>43</v>
       </c>
-      <c r="B43" s="61"/>
-      <c r="C43" s="61"/>
+      <c r="B43" s="62"/>
+      <c r="C43" s="62"/>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A44" s="64" t="s">
         <v>26</v>
       </c>
-      <c r="B44" s="61"/>
-      <c r="C44" s="61"/>
+      <c r="B44" s="62"/>
+      <c r="C44" s="62"/>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A45" s="58"/>
+      <c r="A45" s="60"/>
       <c r="B45" s="59"/>
       <c r="C45" s="59"/>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A46" s="58"/>
+      <c r="A46" s="60"/>
       <c r="B46" s="59"/>
       <c r="C46" s="59"/>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A47" s="58"/>
+      <c r="A47" s="60"/>
       <c r="B47" s="59"/>
       <c r="C47" s="59"/>
     </row>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A24:C24"/>
-    <mergeCell ref="A46:C46"/>
     <mergeCell ref="A47:C47"/>
     <mergeCell ref="A45:C45"/>
     <mergeCell ref="A43:C43"/>
@@ -4316,6 +4422,11 @@
     <mergeCell ref="A33:C33"/>
     <mergeCell ref="A40:C40"/>
     <mergeCell ref="A41:C41"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="A46:C46"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -14520,7 +14631,7 @@
         <v>22</v>
       </c>
       <c r="G191" s="45" t="s">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="H191" s="43" t="s">
         <v>35</v>
@@ -18739,30 +18850,34 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="B1:F86"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+  <dimension ref="B1:J85"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="14" style="6" customWidth="1"/>
     <col min="3" max="3" width="18" style="14" customWidth="1"/>
     <col min="4" max="4" width="24.26953125" style="38" customWidth="1"/>
+    <col min="6" max="6" width="13.453125" customWidth="1"/>
+    <col min="7" max="7" width="25.08984375" customWidth="1"/>
+    <col min="8" max="8" width="29.90625" customWidth="1"/>
+    <col min="11" max="11" width="11.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:6" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="2:8" ht="18.5" x14ac:dyDescent="0.45">
       <c r="B1" s="57" t="s">
         <v>36</v>
       </c>
       <c r="C1" s="56"/>
       <c r="D1" s="56"/>
     </row>
-    <row r="2" spans="2:6" ht="35" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:8" ht="35" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="55" t="s">
         <v>404</v>
       </c>
       <c r="C2" s="56"/>
       <c r="D2" s="56"/>
     </row>
-    <row r="4" spans="2:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:8" ht="45" x14ac:dyDescent="0.35">
       <c r="B4" s="35" t="s">
         <v>28</v>
       </c>
@@ -18772,8 +18887,17 @@
       <c r="D4" s="36" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="5" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="F4" s="69" t="s">
+        <v>528</v>
+      </c>
+      <c r="G4" s="69" t="s">
+        <v>529</v>
+      </c>
+      <c r="H4" s="69" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="5" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B5" s="34" t="s">
         <v>224</v>
       </c>
@@ -18783,16 +18907,17 @@
       <c r="D5" s="37">
         <v>46203</v>
       </c>
-      <c r="E5">
-        <f>_xlfn.XLOOKUP(B5,Table4[ref_id],Table4[euros])</f>
-        <v>20.22</v>
-      </c>
-      <c r="F5">
-        <f>E5*C5</f>
-        <v>3396.96</v>
-      </c>
-    </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="F5" s="70" t="s">
+        <v>531</v>
+      </c>
+      <c r="G5" s="71">
+        <v>165.92526540126542</v>
+      </c>
+      <c r="H5" s="72">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="6" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B6" s="34" t="s">
         <v>229</v>
       </c>
@@ -18802,16 +18927,17 @@
       <c r="D6" s="37">
         <v>46203</v>
       </c>
-      <c r="E6">
-        <f>_xlfn.XLOOKUP(B6,Table4[ref_id],Table4[euros])</f>
-        <v>25.88</v>
-      </c>
-      <c r="F6">
-        <f t="shared" ref="F6:F52" si="0">E6*C6</f>
-        <v>4347.84</v>
-      </c>
-    </row>
-    <row r="7" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="F6" s="70" t="s">
+        <v>532</v>
+      </c>
+      <c r="G6" s="71">
+        <v>241.03174325966435</v>
+      </c>
+      <c r="H6" s="72">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="7" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B7" s="34" t="s">
         <v>372</v>
       </c>
@@ -18821,18 +18947,10 @@
       <c r="D7" s="37">
         <v>46177</v>
       </c>
-      <c r="E7">
-        <f>_xlfn.XLOOKUP(B7,Table4[ref_id],Table4[euros])</f>
-        <v>16.989999999999998</v>
-      </c>
-      <c r="F7">
-        <f t="shared" si="0"/>
-        <v>9786.24</v>
-      </c>
-    </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="8" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B8" s="34" t="s">
-        <v>525</v>
+        <v>521</v>
       </c>
       <c r="C8" s="34">
         <v>140</v>
@@ -18840,16 +18958,8 @@
       <c r="D8" s="37">
         <v>46203</v>
       </c>
-      <c r="E8">
-        <f>_xlfn.XLOOKUP(B8,Table4[ref_id],Table4[euros])</f>
-        <v>19.87</v>
-      </c>
-      <c r="F8">
-        <f t="shared" si="0"/>
-        <v>2781.8</v>
-      </c>
-    </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="9" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B9" s="34" t="s">
         <v>234</v>
       </c>
@@ -18859,16 +18969,8 @@
       <c r="D9" s="37">
         <v>46203</v>
       </c>
-      <c r="E9">
-        <f>_xlfn.XLOOKUP(B9,Table4[ref_id],Table4[euros])</f>
-        <v>17.11</v>
-      </c>
-      <c r="F9">
-        <f t="shared" si="0"/>
-        <v>2395.4</v>
-      </c>
-    </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="10" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B10" s="34" t="s">
         <v>259</v>
       </c>
@@ -18878,16 +18980,8 @@
       <c r="D10" s="37">
         <v>46203</v>
       </c>
-      <c r="E10">
-        <f>_xlfn.XLOOKUP(B10,Table4[ref_id],Table4[euros])</f>
-        <v>21</v>
-      </c>
-      <c r="F10">
-        <f t="shared" si="0"/>
-        <v>6300</v>
-      </c>
-    </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="11" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B11" s="34" t="s">
         <v>374</v>
       </c>
@@ -18897,16 +18991,8 @@
       <c r="D11" s="37">
         <v>46203</v>
       </c>
-      <c r="E11">
-        <f>_xlfn.XLOOKUP(B11,Table4[ref_id],Table4[euros])</f>
-        <v>9.85</v>
-      </c>
-      <c r="F11">
-        <f t="shared" si="0"/>
-        <v>2521.6</v>
-      </c>
-    </row>
-    <row r="12" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="12" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B12" s="34" t="s">
         <v>269</v>
       </c>
@@ -18916,16 +19002,8 @@
       <c r="D12" s="37">
         <v>46203</v>
       </c>
-      <c r="E12">
-        <f>_xlfn.XLOOKUP(B12,Table4[ref_id],Table4[euros])</f>
-        <v>17.260000000000002</v>
-      </c>
-      <c r="F12">
-        <f t="shared" si="0"/>
-        <v>4142.4000000000005</v>
-      </c>
-    </row>
-    <row r="13" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="13" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B13" s="34" t="s">
         <v>306</v>
       </c>
@@ -18935,16 +19013,8 @@
       <c r="D13" s="37">
         <v>46203</v>
       </c>
-      <c r="E13">
-        <f>_xlfn.XLOOKUP(B13,Table4[ref_id],Table4[euros])</f>
-        <v>28.47</v>
-      </c>
-      <c r="F13">
-        <f t="shared" si="0"/>
-        <v>5466.24</v>
-      </c>
-    </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="14" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B14" s="34" t="s">
         <v>318</v>
       </c>
@@ -18954,16 +19024,8 @@
       <c r="D14" s="37">
         <v>46203</v>
       </c>
-      <c r="E14">
-        <f>_xlfn.XLOOKUP(B14,Table4[ref_id],Table4[euros])</f>
-        <v>18.72</v>
-      </c>
-      <c r="F14">
-        <f t="shared" si="0"/>
-        <v>4492.7999999999993</v>
-      </c>
-    </row>
-    <row r="15" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="15" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B15" s="34" t="s">
         <v>322</v>
       </c>
@@ -18973,16 +19035,8 @@
       <c r="D15" s="37">
         <v>46203</v>
       </c>
-      <c r="E15">
-        <f>_xlfn.XLOOKUP(B15,Table4[ref_id],Table4[euros])</f>
-        <v>28.81</v>
-      </c>
-      <c r="F15">
-        <f t="shared" si="0"/>
-        <v>4148.6399999999994</v>
-      </c>
-    </row>
-    <row r="16" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="16" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B16" s="34" t="s">
         <v>337</v>
       </c>
@@ -18992,16 +19046,8 @@
       <c r="D16" s="37">
         <v>46177</v>
       </c>
-      <c r="E16">
-        <f>_xlfn.XLOOKUP(B16,Table4[ref_id],Table4[euros])</f>
-        <v>16.559999999999999</v>
-      </c>
-      <c r="F16">
-        <f t="shared" si="0"/>
-        <v>1788.4799999999998</v>
-      </c>
-    </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="17" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B17" s="34" t="s">
         <v>378</v>
       </c>
@@ -19011,16 +19057,8 @@
       <c r="D17" s="37">
         <v>46203</v>
       </c>
-      <c r="E17">
-        <f>_xlfn.XLOOKUP(B17,Table4[ref_id],Table4[euros])</f>
-        <v>15.67</v>
-      </c>
-      <c r="F17">
-        <f t="shared" si="0"/>
-        <v>6769.44</v>
-      </c>
-    </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="18" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B18" s="34" t="s">
         <v>512</v>
       </c>
@@ -19030,16 +19068,8 @@
       <c r="D18" s="37">
         <v>46203</v>
       </c>
-      <c r="E18">
-        <f>_xlfn.XLOOKUP(B18,Table4[ref_id],Table4[euros])</f>
-        <v>39.58</v>
-      </c>
-      <c r="F18">
-        <f t="shared" si="0"/>
-        <v>3324.72</v>
-      </c>
-    </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="19" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B19" s="34" t="s">
         <v>239</v>
       </c>
@@ -19049,16 +19079,8 @@
       <c r="D19" s="37">
         <v>46203</v>
       </c>
-      <c r="E19">
-        <f>_xlfn.XLOOKUP(B19,Table4[ref_id],Table4[euros])</f>
-        <v>25.4</v>
-      </c>
-      <c r="F19">
-        <f t="shared" si="0"/>
-        <v>2235.1999999999998</v>
-      </c>
-    </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="20" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B20" s="34" t="s">
         <v>242</v>
       </c>
@@ -19068,16 +19090,8 @@
       <c r="D20" s="37">
         <v>46203</v>
       </c>
-      <c r="E20">
-        <f>_xlfn.XLOOKUP(B20,Table4[ref_id],Table4[euros])</f>
-        <v>18.73</v>
-      </c>
-      <c r="F20">
-        <f t="shared" si="0"/>
-        <v>14047.5</v>
-      </c>
-    </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="21" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B21" s="34" t="s">
         <v>243</v>
       </c>
@@ -19087,16 +19101,8 @@
       <c r="D21" s="37">
         <v>46203</v>
       </c>
-      <c r="E21">
-        <f>_xlfn.XLOOKUP(B21,Table4[ref_id],Table4[euros])</f>
-        <v>18.46</v>
-      </c>
-      <c r="F21">
-        <f t="shared" si="0"/>
-        <v>3692</v>
-      </c>
-    </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="22" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B22" s="34" t="s">
         <v>244</v>
       </c>
@@ -19106,16 +19112,8 @@
       <c r="D22" s="37">
         <v>46203</v>
       </c>
-      <c r="E22">
-        <f>_xlfn.XLOOKUP(B22,Table4[ref_id],Table4[euros])</f>
-        <v>19.350000000000001</v>
-      </c>
-      <c r="F22">
-        <f t="shared" si="0"/>
-        <v>1935.0000000000002</v>
-      </c>
-    </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="23" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B23" s="34" t="s">
         <v>245</v>
       </c>
@@ -19125,16 +19123,8 @@
       <c r="D23" s="37">
         <v>46203</v>
       </c>
-      <c r="E23">
-        <f>_xlfn.XLOOKUP(B23,Table4[ref_id],Table4[euros])</f>
-        <v>20.69</v>
-      </c>
-      <c r="F23">
-        <f t="shared" si="0"/>
-        <v>5462.1600000000008</v>
-      </c>
-    </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="24" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B24" s="34" t="s">
         <v>246</v>
       </c>
@@ -19144,16 +19134,8 @@
       <c r="D24" s="37">
         <v>46203</v>
       </c>
-      <c r="E24">
-        <f>_xlfn.XLOOKUP(B24,Table4[ref_id],Table4[euros])</f>
-        <v>19.829999999999998</v>
-      </c>
-      <c r="F24">
-        <f t="shared" si="0"/>
-        <v>951.83999999999992</v>
-      </c>
-    </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="25" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B25" s="34" t="s">
         <v>252</v>
       </c>
@@ -19163,16 +19145,8 @@
       <c r="D25" s="37">
         <v>46203</v>
       </c>
-      <c r="E25">
-        <f>_xlfn.XLOOKUP(B25,Table4[ref_id],Table4[euros])</f>
-        <v>21.47</v>
-      </c>
-      <c r="F25">
-        <f t="shared" si="0"/>
-        <v>1030.56</v>
-      </c>
-    </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="26" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B26" s="34" t="s">
         <v>249</v>
       </c>
@@ -19182,16 +19156,8 @@
       <c r="D26" s="37">
         <v>46203</v>
       </c>
-      <c r="E26">
-        <f>_xlfn.XLOOKUP(B26,Table4[ref_id],Table4[euros])</f>
-        <v>23.11</v>
-      </c>
-      <c r="F26">
-        <f t="shared" si="0"/>
-        <v>2218.56</v>
-      </c>
-    </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="27" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B27" s="34" t="s">
         <v>250</v>
       </c>
@@ -19201,16 +19167,8 @@
       <c r="D27" s="37">
         <v>46203</v>
       </c>
-      <c r="E27">
-        <f>_xlfn.XLOOKUP(B27,Table4[ref_id],Table4[euros])</f>
-        <v>18.52</v>
-      </c>
-      <c r="F27">
-        <f t="shared" si="0"/>
-        <v>3704</v>
-      </c>
-    </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="28" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B28" s="34" t="s">
         <v>251</v>
       </c>
@@ -19220,16 +19178,8 @@
       <c r="D28" s="37">
         <v>46203</v>
       </c>
-      <c r="E28">
-        <f>_xlfn.XLOOKUP(B28,Table4[ref_id],Table4[euros])</f>
-        <v>18.36</v>
-      </c>
-      <c r="F28">
-        <f t="shared" si="0"/>
-        <v>1762.56</v>
-      </c>
-    </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="29" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B29" s="34" t="s">
         <v>521</v>
       </c>
@@ -19239,16 +19189,8 @@
       <c r="D29" s="37">
         <v>46203</v>
       </c>
-      <c r="E29">
-        <f>_xlfn.XLOOKUP(B29,Table4[ref_id],Table4[euros])</f>
-        <v>16.78</v>
-      </c>
-      <c r="F29">
-        <f t="shared" si="0"/>
-        <v>3221.76</v>
-      </c>
-    </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="30" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B30" s="34" t="s">
         <v>279</v>
       </c>
@@ -19258,16 +19200,8 @@
       <c r="D30" s="37">
         <v>46203</v>
       </c>
-      <c r="E30">
-        <f>_xlfn.XLOOKUP(B30,Table4[ref_id],Table4[euros])</f>
-        <v>16.850000000000001</v>
-      </c>
-      <c r="F30">
-        <f t="shared" si="0"/>
-        <v>3370.0000000000005</v>
-      </c>
-    </row>
-    <row r="31" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="31" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B31" s="34" t="s">
         <v>286</v>
       </c>
@@ -19277,16 +19211,8 @@
       <c r="D31" s="37">
         <v>46203</v>
       </c>
-      <c r="E31">
-        <f>_xlfn.XLOOKUP(B31,Table4[ref_id],Table4[euros])</f>
-        <v>17.73</v>
-      </c>
-      <c r="F31">
-        <f t="shared" si="0"/>
-        <v>3546</v>
-      </c>
-    </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="32" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B32" s="34" t="s">
         <v>291</v>
       </c>
@@ -19296,16 +19222,8 @@
       <c r="D32" s="37">
         <v>46203</v>
       </c>
-      <c r="E32">
-        <f>_xlfn.XLOOKUP(B32,Table4[ref_id],Table4[euros])</f>
-        <v>21</v>
-      </c>
-      <c r="F32">
-        <f t="shared" si="0"/>
-        <v>2520</v>
-      </c>
-    </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="33" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B33" s="34" t="s">
         <v>297</v>
       </c>
@@ -19315,16 +19233,8 @@
       <c r="D33" s="37">
         <v>46203</v>
       </c>
-      <c r="E33">
-        <f>_xlfn.XLOOKUP(B33,Table4[ref_id],Table4[euros])</f>
-        <v>21.88</v>
-      </c>
-      <c r="F33">
-        <f t="shared" si="0"/>
-        <v>8752</v>
-      </c>
-    </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="34" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B34" s="34" t="s">
         <v>300</v>
       </c>
@@ -19334,16 +19244,8 @@
       <c r="D34" s="37">
         <v>46203</v>
       </c>
-      <c r="E34">
-        <f>_xlfn.XLOOKUP(B34,Table4[ref_id],Table4[euros])</f>
-        <v>19.8</v>
-      </c>
-      <c r="F34">
-        <f t="shared" si="0"/>
-        <v>4752</v>
-      </c>
-    </row>
-    <row r="35" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="35" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B35" s="34" t="s">
         <v>308</v>
       </c>
@@ -19353,16 +19255,8 @@
       <c r="D35" s="37">
         <v>46203</v>
       </c>
-      <c r="E35">
-        <f>_xlfn.XLOOKUP(B35,Table4[ref_id],Table4[euros])</f>
-        <v>22.97</v>
-      </c>
-      <c r="F35">
-        <f t="shared" si="0"/>
-        <v>2205.12</v>
-      </c>
-    </row>
-    <row r="36" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="36" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B36" s="34" t="s">
         <v>310</v>
       </c>
@@ -19372,16 +19266,8 @@
       <c r="D36" s="37">
         <v>46203</v>
       </c>
-      <c r="E36">
-        <f>_xlfn.XLOOKUP(B36,Table4[ref_id],Table4[euros])</f>
-        <v>32.17</v>
-      </c>
-      <c r="F36">
-        <f t="shared" si="0"/>
-        <v>3860.4</v>
-      </c>
-    </row>
-    <row r="37" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="37" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B37" s="34" t="s">
         <v>513</v>
       </c>
@@ -19391,16 +19277,8 @@
       <c r="D37" s="37">
         <v>46203</v>
       </c>
-      <c r="E37">
-        <f>_xlfn.XLOOKUP(B37,Table4[ref_id],Table4[euros])</f>
-        <v>12.05</v>
-      </c>
-      <c r="F37">
-        <f t="shared" si="0"/>
-        <v>3084.8</v>
-      </c>
-    </row>
-    <row r="38" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="38" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B38" s="34" t="s">
         <v>312</v>
       </c>
@@ -19410,16 +19288,8 @@
       <c r="D38" s="37">
         <v>46203</v>
       </c>
-      <c r="E38">
-        <f>_xlfn.XLOOKUP(B38,Table4[ref_id],Table4[euros])</f>
-        <v>15.16</v>
-      </c>
-      <c r="F38">
-        <f t="shared" si="0"/>
-        <v>2364.96</v>
-      </c>
-    </row>
-    <row r="39" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="39" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B39" s="34" t="s">
         <v>327</v>
       </c>
@@ -19429,16 +19299,8 @@
       <c r="D39" s="37">
         <v>46203</v>
       </c>
-      <c r="E39">
-        <f>_xlfn.XLOOKUP(B39,Table4[ref_id],Table4[euros])</f>
-        <v>8.98</v>
-      </c>
-      <c r="F39">
-        <f t="shared" si="0"/>
-        <v>1077.6000000000001</v>
-      </c>
-    </row>
-    <row r="40" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="40" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B40" s="34" t="s">
         <v>358</v>
       </c>
@@ -19448,16 +19310,8 @@
       <c r="D40" s="37">
         <v>46203</v>
       </c>
-      <c r="E40">
-        <f>_xlfn.XLOOKUP(B40,Table4[ref_id],Table4[euros])</f>
-        <v>32.32</v>
-      </c>
-      <c r="F40">
-        <f t="shared" si="0"/>
-        <v>9308.16</v>
-      </c>
-    </row>
-    <row r="41" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="41" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B41" s="34" t="s">
         <v>359</v>
       </c>
@@ -19467,16 +19321,8 @@
       <c r="D41" s="37">
         <v>46203</v>
       </c>
-      <c r="E41">
-        <f>_xlfn.XLOOKUP(B41,Table4[ref_id],Table4[euros])</f>
-        <v>30.59</v>
-      </c>
-      <c r="F41">
-        <f t="shared" si="0"/>
-        <v>4404.96</v>
-      </c>
-    </row>
-    <row r="42" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="42" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B42" s="34" t="s">
         <v>361</v>
       </c>
@@ -19486,16 +19332,8 @@
       <c r="D42" s="37">
         <v>46203</v>
       </c>
-      <c r="E42">
-        <f>_xlfn.XLOOKUP(B42,Table4[ref_id],Table4[euros])</f>
-        <v>31.03</v>
-      </c>
-      <c r="F42">
-        <f t="shared" si="0"/>
-        <v>4468.32</v>
-      </c>
-    </row>
-    <row r="43" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="43" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B43" s="34" t="s">
         <v>280</v>
       </c>
@@ -19505,16 +19343,8 @@
       <c r="D43" s="37">
         <v>46203</v>
       </c>
-      <c r="E43">
-        <f>_xlfn.XLOOKUP(B43,Table4[ref_id],Table4[euros])</f>
-        <v>22.94</v>
-      </c>
-      <c r="F43">
-        <f t="shared" si="0"/>
-        <v>5505.6</v>
-      </c>
-    </row>
-    <row r="44" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="44" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B44" s="34" t="s">
         <v>365</v>
       </c>
@@ -19524,16 +19354,8 @@
       <c r="D44" s="37">
         <v>46175</v>
       </c>
-      <c r="E44">
-        <f>_xlfn.XLOOKUP(B44,Table4[ref_id],Table4[euros])</f>
-        <v>26.32</v>
-      </c>
-      <c r="F44">
-        <f t="shared" si="0"/>
-        <v>4632.32</v>
-      </c>
-    </row>
-    <row r="45" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="45" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B45" s="34" t="s">
         <v>369</v>
       </c>
@@ -19543,16 +19365,8 @@
       <c r="D45" s="37">
         <v>46203</v>
       </c>
-      <c r="E45">
-        <f>_xlfn.XLOOKUP(B45,Table4[ref_id],Table4[euros])</f>
-        <v>26.32</v>
-      </c>
-      <c r="F45">
-        <f t="shared" si="0"/>
-        <v>2316.16</v>
-      </c>
-    </row>
-    <row r="46" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="46" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B46" s="34" t="s">
         <v>370</v>
       </c>
@@ -19562,16 +19376,8 @@
       <c r="D46" s="37">
         <v>46177</v>
       </c>
-      <c r="E46">
-        <f>_xlfn.XLOOKUP(B46,Table4[ref_id],Table4[euros])</f>
-        <v>23.46</v>
-      </c>
-      <c r="F46">
-        <f t="shared" si="0"/>
-        <v>2064.48</v>
-      </c>
-    </row>
-    <row r="47" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="47" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B47" s="34" t="s">
         <v>371</v>
       </c>
@@ -19581,16 +19387,8 @@
       <c r="D47" s="37">
         <v>46177</v>
       </c>
-      <c r="E47">
-        <f>_xlfn.XLOOKUP(B47,Table4[ref_id],Table4[euros])</f>
-        <v>33.42</v>
-      </c>
-      <c r="F47">
-        <f t="shared" si="0"/>
-        <v>11763.84</v>
-      </c>
-    </row>
-    <row r="48" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="48" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B48" s="34" t="s">
         <v>301</v>
       </c>
@@ -19600,16 +19398,8 @@
       <c r="D48" s="37">
         <v>46177</v>
       </c>
-      <c r="E48">
-        <f>_xlfn.XLOOKUP(B48,Table4[ref_id],Table4[euros])</f>
-        <v>35.36</v>
-      </c>
-      <c r="F48">
-        <f t="shared" si="0"/>
-        <v>6223.36</v>
-      </c>
-    </row>
-    <row r="49" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="49" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B49" s="34" t="s">
         <v>313</v>
       </c>
@@ -19619,16 +19409,8 @@
       <c r="D49" s="37">
         <v>46177</v>
       </c>
-      <c r="E49">
-        <f>_xlfn.XLOOKUP(B49,Table4[ref_id],Table4[euros])</f>
-        <v>17.22</v>
-      </c>
-      <c r="F49">
-        <f t="shared" si="0"/>
-        <v>3306.24</v>
-      </c>
-    </row>
-    <row r="50" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="50" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B50" s="34" t="s">
         <v>253</v>
       </c>
@@ -19638,16 +19420,8 @@
       <c r="D50" s="37">
         <v>46177</v>
       </c>
-      <c r="E50">
-        <f>_xlfn.XLOOKUP(B50,Table4[ref_id],Table4[euros])</f>
-        <v>19.37</v>
-      </c>
-      <c r="F50">
-        <f t="shared" si="0"/>
-        <v>1220.3100000000002</v>
-      </c>
-    </row>
-    <row r="51" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="51" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B51" s="34" t="s">
         <v>377</v>
       </c>
@@ -19657,16 +19431,8 @@
       <c r="D51" s="37">
         <v>46177</v>
       </c>
-      <c r="E51">
-        <f>_xlfn.XLOOKUP(B51,Table4[ref_id],Table4[euros])</f>
-        <v>25.39</v>
-      </c>
-      <c r="F51">
-        <f t="shared" si="0"/>
-        <v>4468.6400000000003</v>
-      </c>
-    </row>
-    <row r="52" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="52" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B52" s="34" t="s">
         <v>314</v>
       </c>
@@ -19676,16 +19442,8 @@
       <c r="D52" s="37">
         <v>46177</v>
       </c>
-      <c r="E52">
-        <f>_xlfn.XLOOKUP(B52,Table4[ref_id],Table4[euros])</f>
-        <v>13.65</v>
-      </c>
-      <c r="F52">
-        <f t="shared" si="0"/>
-        <v>3439.8</v>
-      </c>
-    </row>
-    <row r="53" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="53" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B53" s="34" t="s">
         <v>236</v>
       </c>
@@ -19695,16 +19453,8 @@
       <c r="D53" s="37">
         <v>46195</v>
       </c>
-      <c r="E53">
-        <f>_xlfn.XLOOKUP(B53,Table4[ref_id],Table4[euros])</f>
-        <v>22.36</v>
-      </c>
-      <c r="F53">
-        <f t="shared" ref="F53:F86" si="1">E53*C53</f>
-        <v>4293.12</v>
-      </c>
-    </row>
-    <row r="54" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="54" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B54" s="37" t="s">
         <v>241</v>
       </c>
@@ -19714,16 +19464,8 @@
       <c r="D54" s="37">
         <v>46203</v>
       </c>
-      <c r="E54">
-        <f>_xlfn.XLOOKUP(B54,Table4[ref_id],Table4[euros])</f>
-        <v>22.79</v>
-      </c>
-      <c r="F54">
-        <f t="shared" si="1"/>
-        <v>2187.84</v>
-      </c>
-    </row>
-    <row r="55" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="55" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B55" s="37" t="s">
         <v>254</v>
       </c>
@@ -19733,265 +19475,153 @@
       <c r="D55" s="37">
         <v>46203</v>
       </c>
-      <c r="E55">
-        <f>_xlfn.XLOOKUP(B55,Table4[ref_id],Table4[euros])</f>
-        <v>23</v>
-      </c>
-      <c r="F55">
-        <f t="shared" si="1"/>
-        <v>1449</v>
-      </c>
-    </row>
-    <row r="56" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="56" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B56" s="37" t="s">
-        <v>379</v>
+        <v>255</v>
       </c>
       <c r="C56" s="54">
-        <v>0</v>
+        <v>260</v>
       </c>
       <c r="D56" s="37">
+        <v>46202</v>
+      </c>
+    </row>
+    <row r="57" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B57" s="37" t="s">
+        <v>260</v>
+      </c>
+      <c r="C57" s="54">
+        <v>3808</v>
+      </c>
+      <c r="D57" s="37">
+        <v>46178</v>
+      </c>
+    </row>
+    <row r="58" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B58" s="37" t="s">
+        <v>376</v>
+      </c>
+      <c r="C58" s="54">
+        <v>3060</v>
+      </c>
+      <c r="D58" s="37">
+        <v>46186</v>
+      </c>
+    </row>
+    <row r="59" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B59" s="37" t="s">
+        <v>287</v>
+      </c>
+      <c r="C59" s="54">
+        <v>96</v>
+      </c>
+      <c r="D59" s="37">
         <v>46203</v>
       </c>
-      <c r="E56">
-        <f>_xlfn.XLOOKUP(B56,Table4[ref_id],Table4[euros])</f>
-        <v>17.02</v>
-      </c>
-      <c r="F56">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B57" s="37" t="s">
-        <v>255</v>
-      </c>
-      <c r="C57" s="54">
-        <v>260</v>
-      </c>
-      <c r="D57" s="37">
-        <v>46202</v>
-      </c>
-      <c r="E57">
-        <f>_xlfn.XLOOKUP(B57,Table4[ref_id],Table4[euros])</f>
-        <v>19.59</v>
-      </c>
-      <c r="F57">
-        <f t="shared" si="1"/>
-        <v>5093.3999999999996</v>
-      </c>
-    </row>
-    <row r="58" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B58" s="37" t="s">
-        <v>260</v>
-      </c>
-      <c r="C58" s="54">
-        <v>3808</v>
-      </c>
-      <c r="D58" s="37">
-        <v>46178</v>
-      </c>
-      <c r="E58">
-        <f>_xlfn.XLOOKUP(B58,Table4[ref_id],Table4[euros])</f>
-        <v>22.6</v>
-      </c>
-      <c r="F58">
-        <f t="shared" si="1"/>
-        <v>86060.800000000003</v>
-      </c>
-    </row>
-    <row r="59" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B59" s="37" t="s">
-        <v>376</v>
-      </c>
-      <c r="C59" s="54">
-        <v>3060</v>
-      </c>
-      <c r="D59" s="37">
-        <v>46186</v>
-      </c>
-      <c r="E59">
-        <f>_xlfn.XLOOKUP(B59,Table4[ref_id],Table4[euros])</f>
-        <v>28.96</v>
-      </c>
-      <c r="F59">
-        <f t="shared" si="1"/>
-        <v>88617.600000000006</v>
-      </c>
-    </row>
-    <row r="60" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="60" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B60" s="37" t="s">
-        <v>287</v>
+        <v>298</v>
       </c>
       <c r="C60" s="54">
         <v>96</v>
       </c>
       <c r="D60" s="37">
-        <v>46203</v>
-      </c>
-      <c r="E60">
-        <f>_xlfn.XLOOKUP(B60,Table4[ref_id],Table4[euros])</f>
-        <v>33.74</v>
-      </c>
-      <c r="F60">
-        <f t="shared" si="1"/>
-        <v>3239.04</v>
-      </c>
-    </row>
-    <row r="61" spans="2:6" x14ac:dyDescent="0.35">
+        <v>46177</v>
+      </c>
+    </row>
+    <row r="61" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B61" s="37" t="s">
-        <v>298</v>
+        <v>305</v>
       </c>
       <c r="C61" s="54">
-        <v>96</v>
+        <v>192</v>
       </c>
       <c r="D61" s="37">
         <v>46177</v>
       </c>
-      <c r="E61">
-        <f>_xlfn.XLOOKUP(B61,Table4[ref_id],Table4[euros])</f>
-        <v>40.64</v>
-      </c>
-      <c r="F61">
-        <f t="shared" si="1"/>
-        <v>3901.44</v>
-      </c>
-    </row>
-    <row r="62" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="62" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B62" s="37" t="s">
-        <v>305</v>
+        <v>261</v>
       </c>
       <c r="C62" s="54">
-        <v>192</v>
+        <v>64</v>
       </c>
       <c r="D62" s="37">
         <v>46177</v>
       </c>
-      <c r="E62">
-        <f>_xlfn.XLOOKUP(B62,Table4[ref_id],Table4[euros])</f>
-        <v>30.94</v>
-      </c>
-      <c r="F62">
-        <f t="shared" si="1"/>
-        <v>5940.4800000000005</v>
-      </c>
-    </row>
-    <row r="63" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="63" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B63" s="37" t="s">
-        <v>261</v>
+        <v>328</v>
       </c>
       <c r="C63" s="54">
-        <v>64</v>
+        <v>96</v>
       </c>
       <c r="D63" s="37">
-        <v>46177</v>
-      </c>
-      <c r="E63">
-        <f>_xlfn.XLOOKUP(B63,Table4[ref_id],Table4[euros])</f>
-        <v>40.479999999999997</v>
-      </c>
-      <c r="F63">
-        <f t="shared" si="1"/>
-        <v>2590.7199999999998</v>
-      </c>
-    </row>
-    <row r="64" spans="2:6" x14ac:dyDescent="0.35">
+        <v>46175</v>
+      </c>
+    </row>
+    <row r="64" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B64" s="37" t="s">
-        <v>328</v>
+        <v>265</v>
       </c>
       <c r="C64" s="54">
-        <v>96</v>
+        <v>256</v>
       </c>
       <c r="D64" s="37">
-        <v>46175</v>
-      </c>
-      <c r="E64">
-        <f>_xlfn.XLOOKUP(B64,Table4[ref_id],Table4[euros])</f>
-        <v>37.94</v>
-      </c>
-      <c r="F64">
-        <f t="shared" si="1"/>
-        <v>3642.24</v>
-      </c>
-    </row>
-    <row r="65" spans="2:6" x14ac:dyDescent="0.35">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="65" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B65" s="37" t="s">
-        <v>265</v>
+        <v>352</v>
       </c>
       <c r="C65" s="54">
-        <v>256</v>
+        <v>600</v>
       </c>
       <c r="D65" s="37">
         <v>46203</v>
       </c>
-      <c r="E65">
-        <f>_xlfn.XLOOKUP(B65,Table4[ref_id],Table4[euros])</f>
-        <v>6.71</v>
-      </c>
-      <c r="F65">
-        <f t="shared" si="1"/>
-        <v>1717.76</v>
-      </c>
-    </row>
-    <row r="66" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="66" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B66" s="37" t="s">
-        <v>352</v>
+        <v>341</v>
       </c>
       <c r="C66" s="54">
-        <v>600</v>
+        <v>216</v>
       </c>
       <c r="D66" s="37">
         <v>46203</v>
       </c>
-      <c r="E66">
-        <f>_xlfn.XLOOKUP(B66,Table4[ref_id],Table4[euros])</f>
-        <v>11.34</v>
-      </c>
-      <c r="F66">
-        <f t="shared" si="1"/>
-        <v>6804</v>
-      </c>
-    </row>
-    <row r="67" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="67" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B67" s="37" t="s">
-        <v>341</v>
+        <v>348</v>
       </c>
       <c r="C67" s="54">
-        <v>216</v>
+        <v>108</v>
       </c>
       <c r="D67" s="37">
         <v>46203</v>
       </c>
-      <c r="E67">
-        <f>_xlfn.XLOOKUP(B67,Table4[ref_id],Table4[euros])</f>
-        <v>17.28</v>
-      </c>
-      <c r="F67">
-        <f t="shared" si="1"/>
-        <v>3732.4800000000005</v>
-      </c>
-    </row>
-    <row r="68" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="68" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B68" s="37" t="s">
-        <v>348</v>
+        <v>362</v>
       </c>
       <c r="C68" s="54">
-        <v>108</v>
+        <v>72</v>
       </c>
       <c r="D68" s="37">
         <v>46203</v>
       </c>
-      <c r="E68">
-        <f>_xlfn.XLOOKUP(B68,Table4[ref_id],Table4[euros])</f>
-        <v>16.489999999999998</v>
-      </c>
-      <c r="F68">
-        <f t="shared" si="1"/>
-        <v>1780.9199999999998</v>
-      </c>
-    </row>
-    <row r="69" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="69" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B69" s="37" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="C69" s="54">
         <v>72</v>
@@ -19999,94 +19629,54 @@
       <c r="D69" s="37">
         <v>46203</v>
       </c>
-      <c r="E69">
-        <f>_xlfn.XLOOKUP(B69,Table4[ref_id],Table4[euros])</f>
-        <v>32.81</v>
-      </c>
-      <c r="F69">
-        <f t="shared" si="1"/>
-        <v>2362.3200000000002</v>
-      </c>
-    </row>
-    <row r="70" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="70" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B70" s="37" t="s">
-        <v>364</v>
+        <v>321</v>
       </c>
       <c r="C70" s="54">
-        <v>72</v>
+        <v>360</v>
       </c>
       <c r="D70" s="37">
         <v>46203</v>
       </c>
-      <c r="E70">
-        <f>_xlfn.XLOOKUP(B70,Table4[ref_id],Table4[euros])</f>
-        <v>32.35</v>
-      </c>
-      <c r="F70">
-        <f t="shared" si="1"/>
-        <v>2329.2000000000003</v>
-      </c>
-    </row>
-    <row r="71" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="71" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B71" s="37" t="s">
-        <v>321</v>
+        <v>375</v>
       </c>
       <c r="C71" s="54">
-        <v>360</v>
+        <v>384</v>
       </c>
       <c r="D71" s="37">
         <v>46203</v>
       </c>
-      <c r="E71">
-        <f>_xlfn.XLOOKUP(B71,Table4[ref_id],Table4[euros])</f>
-        <v>30.98</v>
-      </c>
-      <c r="F71">
-        <f t="shared" si="1"/>
-        <v>11152.8</v>
-      </c>
-    </row>
-    <row r="72" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="72" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B72" s="37" t="s">
-        <v>375</v>
+        <v>307</v>
       </c>
       <c r="C72" s="54">
-        <v>384</v>
+        <v>192</v>
       </c>
       <c r="D72" s="37">
         <v>46203</v>
       </c>
-      <c r="E72">
-        <f>_xlfn.XLOOKUP(B72,Table4[ref_id],Table4[euros])</f>
-        <v>15.68</v>
-      </c>
-      <c r="F72">
-        <f t="shared" si="1"/>
-        <v>6021.12</v>
-      </c>
-    </row>
-    <row r="73" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="73" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B73" s="37" t="s">
-        <v>307</v>
+        <v>293</v>
       </c>
       <c r="C73" s="54">
-        <v>192</v>
+        <v>63</v>
       </c>
       <c r="D73" s="37">
         <v>46203</v>
       </c>
-      <c r="E73">
-        <f>_xlfn.XLOOKUP(B73,Table4[ref_id],Table4[euros])</f>
-        <v>30.94</v>
-      </c>
-      <c r="F73">
-        <f t="shared" si="1"/>
-        <v>5940.4800000000005</v>
-      </c>
-    </row>
-    <row r="74" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="74" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B74" s="37" t="s">
-        <v>293</v>
+        <v>282</v>
       </c>
       <c r="C74" s="54">
         <v>63</v>
@@ -20094,18 +19684,10 @@
       <c r="D74" s="37">
         <v>46203</v>
       </c>
-      <c r="E74">
-        <f>_xlfn.XLOOKUP(B74,Table4[ref_id],Table4[euros])</f>
-        <v>14.71</v>
-      </c>
-      <c r="F74">
-        <f t="shared" si="1"/>
-        <v>926.73</v>
-      </c>
-    </row>
-    <row r="75" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="75" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B75" s="37" t="s">
-        <v>282</v>
+        <v>333</v>
       </c>
       <c r="C75" s="54">
         <v>63</v>
@@ -20113,222 +19695,115 @@
       <c r="D75" s="37">
         <v>46203</v>
       </c>
-      <c r="E75">
-        <f>_xlfn.XLOOKUP(B75,Table4[ref_id],Table4[euros])</f>
-        <v>16.309999999999999</v>
-      </c>
-      <c r="F75">
-        <f t="shared" si="1"/>
-        <v>1027.53</v>
-      </c>
-    </row>
-    <row r="76" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="76" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B76" s="37" t="s">
-        <v>333</v>
+        <v>325</v>
       </c>
       <c r="C76" s="54">
-        <v>63</v>
+        <v>1276</v>
       </c>
       <c r="D76" s="37">
         <v>46203</v>
       </c>
-      <c r="E76">
-        <f>_xlfn.XLOOKUP(B76,Table4[ref_id],Table4[euros])</f>
-        <v>16.93</v>
-      </c>
-      <c r="F76">
-        <f t="shared" si="1"/>
-        <v>1066.5899999999999</v>
-      </c>
-    </row>
-    <row r="77" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="77" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B77" s="37" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="C77" s="54">
-        <v>1276</v>
+        <v>768</v>
       </c>
       <c r="D77" s="37">
         <v>46203</v>
       </c>
-      <c r="E77">
-        <f>_xlfn.XLOOKUP(B77,Table4[ref_id],Table4[euros])</f>
-        <v>8.8000000000000007</v>
-      </c>
-      <c r="F77">
-        <f t="shared" si="1"/>
-        <v>11228.800000000001</v>
-      </c>
-    </row>
-    <row r="78" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="78" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B78" s="37" t="s">
-        <v>326</v>
+        <v>296</v>
       </c>
       <c r="C78" s="54">
-        <v>768</v>
+        <v>896</v>
       </c>
       <c r="D78" s="37">
         <v>46203</v>
       </c>
-      <c r="E78">
-        <f>_xlfn.XLOOKUP(B78,Table4[ref_id],Table4[euros])</f>
-        <v>9.34</v>
-      </c>
-      <c r="F78">
-        <f t="shared" si="1"/>
-        <v>7173.12</v>
-      </c>
-    </row>
-    <row r="79" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="79" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B79" s="37" t="s">
-        <v>296</v>
+        <v>329</v>
       </c>
       <c r="C79" s="54">
-        <v>896</v>
+        <v>256</v>
       </c>
       <c r="D79" s="37">
         <v>46203</v>
       </c>
-      <c r="E79">
-        <f>_xlfn.XLOOKUP(B79,Table4[ref_id],Table4[euros])</f>
-        <v>8.9700000000000006</v>
-      </c>
-      <c r="F79">
-        <f t="shared" si="1"/>
-        <v>8037.1200000000008</v>
-      </c>
-    </row>
-    <row r="80" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="80" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B80" s="37" t="s">
-        <v>329</v>
+        <v>223</v>
       </c>
       <c r="C80" s="54">
-        <v>256</v>
+        <v>88</v>
       </c>
       <c r="D80" s="37">
         <v>46203</v>
       </c>
-      <c r="E80">
-        <f>_xlfn.XLOOKUP(B80,Table4[ref_id],Table4[euros])</f>
-        <v>8.9700000000000006</v>
-      </c>
-      <c r="F80">
-        <f t="shared" si="1"/>
-        <v>2296.3200000000002</v>
-      </c>
-    </row>
-    <row r="81" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="81" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B81" s="37" t="s">
-        <v>223</v>
+        <v>330</v>
       </c>
       <c r="C81" s="54">
-        <v>88</v>
+        <v>112</v>
       </c>
       <c r="D81" s="37">
         <v>46203</v>
       </c>
-      <c r="E81">
-        <f>_xlfn.XLOOKUP(B81,Table4[ref_id],Table4[euros])</f>
-        <v>23.46</v>
-      </c>
-      <c r="F81">
-        <f t="shared" si="1"/>
-        <v>2064.48</v>
-      </c>
-    </row>
-    <row r="82" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="82" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B82" s="37" t="s">
-        <v>330</v>
+        <v>226</v>
       </c>
       <c r="C82" s="54">
-        <v>112</v>
+        <v>84</v>
       </c>
       <c r="D82" s="37">
         <v>46203</v>
       </c>
-      <c r="E82">
-        <f>_xlfn.XLOOKUP(B82,Table4[ref_id],Table4[euros])</f>
-        <v>10.06</v>
-      </c>
-      <c r="F82">
-        <f t="shared" si="1"/>
-        <v>1126.72</v>
-      </c>
-    </row>
-    <row r="83" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="83" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B83" s="37" t="s">
-        <v>226</v>
+        <v>270</v>
       </c>
       <c r="C83" s="54">
-        <v>84</v>
+        <v>72</v>
       </c>
       <c r="D83" s="37">
         <v>46203</v>
       </c>
-      <c r="E83">
-        <f>_xlfn.XLOOKUP(B83,Table4[ref_id],Table4[euros])</f>
-        <v>21.61</v>
-      </c>
-      <c r="F83">
-        <f t="shared" si="1"/>
-        <v>1815.24</v>
-      </c>
-    </row>
-    <row r="84" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="84" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B84" s="37" t="s">
-        <v>270</v>
+        <v>288</v>
       </c>
       <c r="C84" s="54">
-        <v>72</v>
+        <v>48</v>
       </c>
       <c r="D84" s="37">
         <v>46203</v>
       </c>
-      <c r="E84">
-        <f>_xlfn.XLOOKUP(B84,Table4[ref_id],Table4[euros])</f>
-        <v>25.29</v>
-      </c>
-      <c r="F84">
-        <f t="shared" si="1"/>
-        <v>1820.8799999999999</v>
-      </c>
-    </row>
-    <row r="85" spans="2:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="85" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B85" s="37" t="s">
-        <v>288</v>
+        <v>225</v>
       </c>
       <c r="C85" s="54">
-        <v>48</v>
+        <v>84</v>
       </c>
       <c r="D85" s="37">
         <v>46203</v>
-      </c>
-      <c r="E85">
-        <f>_xlfn.XLOOKUP(B85,Table4[ref_id],Table4[euros])</f>
-        <v>37.49</v>
-      </c>
-      <c r="F85">
-        <f t="shared" si="1"/>
-        <v>1799.52</v>
-      </c>
-    </row>
-    <row r="86" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B86" s="37" t="s">
-        <v>225</v>
-      </c>
-      <c r="C86" s="54">
-        <v>84</v>
-      </c>
-      <c r="D86" s="37">
-        <v>46203</v>
-      </c>
-      <c r="E86">
-        <f>_xlfn.XLOOKUP(B86,Table4[ref_id],Table4[euros])</f>
-        <v>21</v>
-      </c>
-      <c r="F86">
-        <f t="shared" si="1"/>
-        <v>1764</v>
       </c>
     </row>
   </sheetData>
@@ -20337,6 +19812,7 @@
     <mergeCell ref="B1:D1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add Optuna figure generation script and result CSV files
- Created `generate_optuna_figures.py` to generate and save various visualizations from Optuna study results.
- Added `results_mutation_rate_normalised.csv` containing mutation rate analysis data.
- Added `results_population_size_normalised.csv` containing population size analysis data.
- Included a temporary Excel file `Inputs_EmpresaX.xlsx` for input data.
</commit_message>
<xml_diff>
--- a/Inputs_EmpresaX.xlsx
+++ b/Inputs_EmpresaX.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kaizen\Documents\tese\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00E759BB-FC63-4BE4-B76D-641271111F37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B12E16C-4855-47FC-B1D2-AFB9806C9D41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2891,6 +2891,18 @@
     <xf numFmtId="1" fontId="6" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="21" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2900,16 +2912,16 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2927,33 +2939,11 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="21" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="21">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="20">
     <dxf>
       <font>
         <b val="0"/>
@@ -3692,26 +3682,26 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{A2E0425D-8D3D-4317-A507-ADC777C31517}" name="Table4" displayName="Table4" ref="A4:Q192" totalsRowShown="0" headerRowDxfId="20" dataDxfId="19" tableBorderDxfId="18">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{A2E0425D-8D3D-4317-A507-ADC777C31517}" name="Table4" displayName="Table4" ref="A4:Q192" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18" tableBorderDxfId="17">
   <autoFilter ref="A4:Q192" xr:uid="{A2E0425D-8D3D-4317-A507-ADC777C31517}"/>
   <tableColumns count="17">
-    <tableColumn id="1" xr3:uid="{26D481BD-1A66-4F75-A5DB-835BDEAD35EC}" name="ref_id" dataDxfId="17"/>
-    <tableColumn id="2" xr3:uid="{AF3D888D-29CC-4818-9F37-35E1C095FEBC}" name="nome" dataDxfId="16"/>
-    <tableColumn id="21" xr3:uid="{A36D18E5-0E2F-48D2-A9EA-1667409CF7FA}" name="Unid_caixa" dataDxfId="15"/>
-    <tableColumn id="19" xr3:uid="{901BF69A-B9CB-436F-8A73-E52E627A4C44}" name="nao_produzir_segunda" dataDxfId="14"/>
-    <tableColumn id="3" xr3:uid="{73E06642-D2DC-4B3F-B7AE-6A99CF0B73CD}" name="família" dataDxfId="13"/>
-    <tableColumn id="4" xr3:uid="{47F7E5B0-45A6-4E01-8304-DD4D19A9E24E}" name="ativa" dataDxfId="12"/>
-    <tableColumn id="10" xr3:uid="{E576D14B-BDA0-4CA6-B2F4-097D5C1CE99B}" name="pode_L1" dataDxfId="11"/>
-    <tableColumn id="11" xr3:uid="{B29DBEC4-DD50-4914-98AC-30F025559FDC}" name="tempo_L1_prod_min (cadência de L1)" dataDxfId="10"/>
-    <tableColumn id="12" xr3:uid="{14DD02B2-C00E-494B-A8F3-3FFAE31BC4FB}" name="operadores_nec_L1_acab" dataDxfId="9"/>
-    <tableColumn id="13" xr3:uid="{89492EE9-DE84-43EE-B12E-2605FE3EAD79}" name="operadores_nec_L1_prod" dataDxfId="8"/>
-    <tableColumn id="14" xr3:uid="{780BF028-7B4E-42E1-B807-EDB2FB22CEE7}" name="pode_L2" dataDxfId="7"/>
-    <tableColumn id="15" xr3:uid="{FD12F15B-F3BE-48A4-B186-794E71F468D8}" name="tempo_L2_prod_min (cadência de L2)" dataDxfId="6"/>
-    <tableColumn id="16" xr3:uid="{2B695F9C-3774-41DD-8FE4-AF094E98B022}" name="tempo_L2_acab_min (cadência de L2)" dataDxfId="5"/>
-    <tableColumn id="20" xr3:uid="{46C45284-5F2B-442A-A3EB-D66468126784}" name="operadores_nec_L2_acab" dataDxfId="4"/>
-    <tableColumn id="17" xr3:uid="{1453032D-3307-46D2-BB7E-3D55B4D2E43D}" name="operadores_nec_L2_prod" dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{5009F860-773A-42AE-9780-72CCCE321658}" name="kg" dataDxfId="2"/>
-    <tableColumn id="18" xr3:uid="{3939DDEA-30DE-43D1-B600-33ECEC5CD680}" name="euros" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{26D481BD-1A66-4F75-A5DB-835BDEAD35EC}" name="ref_id" dataDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{AF3D888D-29CC-4818-9F37-35E1C095FEBC}" name="nome" dataDxfId="15"/>
+    <tableColumn id="21" xr3:uid="{A36D18E5-0E2F-48D2-A9EA-1667409CF7FA}" name="Unid_caixa" dataDxfId="14"/>
+    <tableColumn id="19" xr3:uid="{901BF69A-B9CB-436F-8A73-E52E627A4C44}" name="nao_produzir_segunda" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{73E06642-D2DC-4B3F-B7AE-6A99CF0B73CD}" name="família" dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{47F7E5B0-45A6-4E01-8304-DD4D19A9E24E}" name="ativa" dataDxfId="11"/>
+    <tableColumn id="10" xr3:uid="{E576D14B-BDA0-4CA6-B2F4-097D5C1CE99B}" name="pode_L1" dataDxfId="10"/>
+    <tableColumn id="11" xr3:uid="{B29DBEC4-DD50-4914-98AC-30F025559FDC}" name="tempo_L1_prod_min (cadência de L1)" dataDxfId="9"/>
+    <tableColumn id="12" xr3:uid="{14DD02B2-C00E-494B-A8F3-3FFAE31BC4FB}" name="operadores_nec_L1_acab" dataDxfId="8"/>
+    <tableColumn id="13" xr3:uid="{89492EE9-DE84-43EE-B12E-2605FE3EAD79}" name="operadores_nec_L1_prod" dataDxfId="7"/>
+    <tableColumn id="14" xr3:uid="{780BF028-7B4E-42E1-B807-EDB2FB22CEE7}" name="pode_L2" dataDxfId="6"/>
+    <tableColumn id="15" xr3:uid="{FD12F15B-F3BE-48A4-B186-794E71F468D8}" name="tempo_L2_prod_min (cadência de L2)" dataDxfId="5"/>
+    <tableColumn id="16" xr3:uid="{2B695F9C-3774-41DD-8FE4-AF094E98B022}" name="tempo_L2_acab_min (cadência de L2)" dataDxfId="4"/>
+    <tableColumn id="20" xr3:uid="{46C45284-5F2B-442A-A3EB-D66468126784}" name="operadores_nec_L2_acab" dataDxfId="3"/>
+    <tableColumn id="17" xr3:uid="{1453032D-3307-46D2-BB7E-3D55B4D2E43D}" name="operadores_nec_L2_prod" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{5009F860-773A-42AE-9780-72CCCE321658}" name="kg" dataDxfId="1"/>
+    <tableColumn id="18" xr3:uid="{3939DDEA-30DE-43D1-B600-33ECEC5CD680}" name="euros" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4058,11 +4048,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A1" s="57" t="s">
+      <c r="A1" s="61" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="56"/>
-      <c r="C1" s="56"/>
+      <c r="B1" s="60"/>
+      <c r="C1" s="60"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
@@ -4094,11 +4084,11 @@
       <c r="C5" s="3"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A6" s="58" t="s">
+      <c r="A6" s="66" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="59"/>
-      <c r="C6" s="59"/>
+      <c r="B6" s="63"/>
+      <c r="C6" s="63"/>
     </row>
     <row r="7" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
@@ -4131,11 +4121,11 @@
       <c r="C9" s="3"/>
     </row>
     <row r="11" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="58" t="s">
+      <c r="A11" s="66" t="s">
         <v>7</v>
       </c>
-      <c r="B11" s="59"/>
-      <c r="C11" s="59"/>
+      <c r="B11" s="63"/>
+      <c r="C11" s="63"/>
     </row>
     <row r="12" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A12" s="7" t="s">
@@ -4159,11 +4149,11 @@
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A15" s="58" t="s">
+      <c r="A15" s="66" t="s">
         <v>9</v>
       </c>
-      <c r="B15" s="59"/>
-      <c r="C15" s="59"/>
+      <c r="B15" s="63"/>
+      <c r="C15" s="63"/>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" s="7" t="s">
@@ -4245,11 +4235,11 @@
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A24" s="58" t="s">
+      <c r="A24" s="66" t="s">
         <v>19</v>
       </c>
-      <c r="B24" s="59"/>
-      <c r="C24" s="59"/>
+      <c r="B24" s="63"/>
+      <c r="C24" s="63"/>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A25" s="7" t="s">
@@ -4329,11 +4319,11 @@
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A33" s="58" t="s">
+      <c r="A33" s="66" t="s">
         <v>21</v>
       </c>
-      <c r="B33" s="59"/>
-      <c r="C33" s="59"/>
+      <c r="B33" s="63"/>
+      <c r="C33" s="63"/>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A34" s="12" t="s">
@@ -4348,69 +4338,74 @@
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A37" s="66" t="s">
+      <c r="A37" s="70" t="s">
         <v>23</v>
       </c>
-      <c r="B37" s="59"/>
-      <c r="C37" s="59"/>
+      <c r="B37" s="63"/>
+      <c r="C37" s="63"/>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A39" s="65" t="s">
+      <c r="A39" s="69" t="s">
         <v>42</v>
       </c>
-      <c r="B39" s="62"/>
-      <c r="C39" s="62"/>
+      <c r="B39" s="65"/>
+      <c r="C39" s="65"/>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A40" s="64" t="s">
+      <c r="A40" s="68" t="s">
         <v>24</v>
       </c>
-      <c r="B40" s="62"/>
-      <c r="C40" s="62"/>
+      <c r="B40" s="65"/>
+      <c r="C40" s="65"/>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A41" s="64"/>
-      <c r="B41" s="62"/>
-      <c r="C41" s="62"/>
+      <c r="A41" s="68"/>
+      <c r="B41" s="65"/>
+      <c r="C41" s="65"/>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A42" s="63" t="s">
+      <c r="A42" s="67" t="s">
         <v>25</v>
       </c>
-      <c r="B42" s="62"/>
-      <c r="C42" s="62"/>
+      <c r="B42" s="65"/>
+      <c r="C42" s="65"/>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A43" s="61" t="s">
+      <c r="A43" s="64" t="s">
         <v>43</v>
       </c>
-      <c r="B43" s="62"/>
-      <c r="C43" s="62"/>
+      <c r="B43" s="65"/>
+      <c r="C43" s="65"/>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A44" s="64" t="s">
+      <c r="A44" s="68" t="s">
         <v>26</v>
       </c>
-      <c r="B44" s="62"/>
-      <c r="C44" s="62"/>
+      <c r="B44" s="65"/>
+      <c r="C44" s="65"/>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A45" s="60"/>
-      <c r="B45" s="59"/>
-      <c r="C45" s="59"/>
+      <c r="A45" s="62"/>
+      <c r="B45" s="63"/>
+      <c r="C45" s="63"/>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A46" s="60"/>
-      <c r="B46" s="59"/>
-      <c r="C46" s="59"/>
+      <c r="A46" s="62"/>
+      <c r="B46" s="63"/>
+      <c r="C46" s="63"/>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A47" s="60"/>
-      <c r="B47" s="59"/>
-      <c r="C47" s="59"/>
+      <c r="A47" s="62"/>
+      <c r="B47" s="63"/>
+      <c r="C47" s="63"/>
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="A46:C46"/>
     <mergeCell ref="A47:C47"/>
     <mergeCell ref="A45:C45"/>
     <mergeCell ref="A43:C43"/>
@@ -4422,11 +4417,6 @@
     <mergeCell ref="A33:C33"/>
     <mergeCell ref="A40:C40"/>
     <mergeCell ref="A41:C41"/>
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A24:C24"/>
-    <mergeCell ref="A46:C46"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4458,44 +4448,44 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A1" s="57" t="s">
+      <c r="A1" s="61" t="s">
         <v>27</v>
       </c>
-      <c r="B1" s="56"/>
-      <c r="C1" s="56"/>
-      <c r="D1" s="56"/>
-      <c r="E1" s="56"/>
-      <c r="F1" s="56"/>
-      <c r="G1" s="56"/>
-      <c r="H1" s="56"/>
-      <c r="I1" s="56"/>
-      <c r="J1" s="56"/>
-      <c r="K1" s="56"/>
-      <c r="L1" s="56"/>
-      <c r="M1" s="56"/>
-      <c r="N1" s="56"/>
-      <c r="O1" s="56"/>
+      <c r="B1" s="60"/>
+      <c r="C1" s="60"/>
+      <c r="D1" s="60"/>
+      <c r="E1" s="60"/>
+      <c r="F1" s="60"/>
+      <c r="G1" s="60"/>
+      <c r="H1" s="60"/>
+      <c r="I1" s="60"/>
+      <c r="J1" s="60"/>
+      <c r="K1" s="60"/>
+      <c r="L1" s="60"/>
+      <c r="M1" s="60"/>
+      <c r="N1" s="60"/>
+      <c r="O1" s="60"/>
     </row>
     <row r="2" spans="1:17" ht="50" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="67" t="s">
+      <c r="A2" s="71" t="s">
         <v>44</v>
       </c>
-      <c r="B2" s="67"/>
-      <c r="C2" s="67"/>
-      <c r="D2" s="67"/>
-      <c r="E2" s="67"/>
-      <c r="F2" s="67"/>
-      <c r="G2" s="67"/>
-      <c r="H2" s="67"/>
-      <c r="I2" s="67"/>
-      <c r="J2" s="67"/>
-      <c r="K2" s="67"/>
-      <c r="L2" s="67"/>
-      <c r="M2" s="67"/>
-      <c r="N2" s="67"/>
-      <c r="O2" s="67"/>
-      <c r="P2" s="67"/>
-      <c r="Q2" s="67"/>
+      <c r="B2" s="71"/>
+      <c r="C2" s="71"/>
+      <c r="D2" s="71"/>
+      <c r="E2" s="71"/>
+      <c r="F2" s="71"/>
+      <c r="G2" s="71"/>
+      <c r="H2" s="71"/>
+      <c r="I2" s="71"/>
+      <c r="J2" s="71"/>
+      <c r="K2" s="71"/>
+      <c r="L2" s="71"/>
+      <c r="M2" s="71"/>
+      <c r="N2" s="71"/>
+      <c r="O2" s="71"/>
+      <c r="P2" s="71"/>
+      <c r="Q2" s="71"/>
     </row>
     <row r="4" spans="1:17" ht="31" x14ac:dyDescent="0.35">
       <c r="A4" s="15" t="s">
@@ -12899,9 +12889,11 @@
         <v>22</v>
       </c>
       <c r="L158" s="45">
-        <v>76</v>
-      </c>
-      <c r="M158" s="45"/>
+        <v>1824</v>
+      </c>
+      <c r="M158" s="45">
+        <v>1824</v>
+      </c>
       <c r="N158" s="45">
         <v>2</v>
       </c>
@@ -14757,109 +14749,109 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A1" s="57" t="s">
+      <c r="A1" s="61" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="56"/>
-      <c r="C1" s="56"/>
-      <c r="D1" s="56"/>
-      <c r="E1" s="56"/>
-      <c r="F1" s="56"/>
-      <c r="G1" s="56"/>
-      <c r="H1" s="56"/>
-      <c r="I1" s="56"/>
-      <c r="J1" s="56"/>
-      <c r="K1" s="56"/>
-      <c r="L1" s="56"/>
-      <c r="M1" s="56"/>
-      <c r="N1" s="56"/>
-      <c r="O1" s="56"/>
-      <c r="P1" s="56"/>
-      <c r="Q1" s="56"/>
-      <c r="R1" s="56"/>
-      <c r="S1" s="56"/>
-      <c r="T1" s="56"/>
-      <c r="U1" s="56"/>
-      <c r="V1" s="56"/>
-      <c r="W1" s="56"/>
-      <c r="X1" s="56"/>
-      <c r="Y1" s="56"/>
-      <c r="Z1" s="56"/>
-      <c r="AA1" s="56"/>
-      <c r="AB1" s="56"/>
-      <c r="AC1" s="56"/>
+      <c r="B1" s="60"/>
+      <c r="C1" s="60"/>
+      <c r="D1" s="60"/>
+      <c r="E1" s="60"/>
+      <c r="F1" s="60"/>
+      <c r="G1" s="60"/>
+      <c r="H1" s="60"/>
+      <c r="I1" s="60"/>
+      <c r="J1" s="60"/>
+      <c r="K1" s="60"/>
+      <c r="L1" s="60"/>
+      <c r="M1" s="60"/>
+      <c r="N1" s="60"/>
+      <c r="O1" s="60"/>
+      <c r="P1" s="60"/>
+      <c r="Q1" s="60"/>
+      <c r="R1" s="60"/>
+      <c r="S1" s="60"/>
+      <c r="T1" s="60"/>
+      <c r="U1" s="60"/>
+      <c r="V1" s="60"/>
+      <c r="W1" s="60"/>
+      <c r="X1" s="60"/>
+      <c r="Y1" s="60"/>
+      <c r="Z1" s="60"/>
+      <c r="AA1" s="60"/>
+      <c r="AB1" s="60"/>
+      <c r="AC1" s="60"/>
     </row>
     <row r="2" spans="1:38" x14ac:dyDescent="0.35">
-      <c r="A2" s="55" t="s">
+      <c r="A2" s="59" t="s">
         <v>400</v>
       </c>
-      <c r="B2" s="56"/>
-      <c r="C2" s="56"/>
-      <c r="D2" s="56"/>
-      <c r="E2" s="56"/>
-      <c r="F2" s="56"/>
-      <c r="G2" s="56"/>
-      <c r="H2" s="56"/>
-      <c r="I2" s="56"/>
-      <c r="J2" s="56"/>
-      <c r="K2" s="56"/>
-      <c r="L2" s="56"/>
-      <c r="M2" s="56"/>
-      <c r="N2" s="56"/>
-      <c r="O2" s="56"/>
-      <c r="P2" s="56"/>
-      <c r="Q2" s="56"/>
-      <c r="R2" s="56"/>
-      <c r="S2" s="56"/>
-      <c r="T2" s="56"/>
-      <c r="U2" s="56"/>
-      <c r="V2" s="56"/>
-      <c r="W2" s="56"/>
-      <c r="X2" s="56"/>
-      <c r="Y2" s="56"/>
-      <c r="Z2" s="56"/>
-      <c r="AA2" s="56"/>
-      <c r="AB2" s="56"/>
-      <c r="AC2" s="56"/>
+      <c r="B2" s="60"/>
+      <c r="C2" s="60"/>
+      <c r="D2" s="60"/>
+      <c r="E2" s="60"/>
+      <c r="F2" s="60"/>
+      <c r="G2" s="60"/>
+      <c r="H2" s="60"/>
+      <c r="I2" s="60"/>
+      <c r="J2" s="60"/>
+      <c r="K2" s="60"/>
+      <c r="L2" s="60"/>
+      <c r="M2" s="60"/>
+      <c r="N2" s="60"/>
+      <c r="O2" s="60"/>
+      <c r="P2" s="60"/>
+      <c r="Q2" s="60"/>
+      <c r="R2" s="60"/>
+      <c r="S2" s="60"/>
+      <c r="T2" s="60"/>
+      <c r="U2" s="60"/>
+      <c r="V2" s="60"/>
+      <c r="W2" s="60"/>
+      <c r="X2" s="60"/>
+      <c r="Y2" s="60"/>
+      <c r="Z2" s="60"/>
+      <c r="AA2" s="60"/>
+      <c r="AB2" s="60"/>
+      <c r="AC2" s="60"/>
     </row>
     <row r="3" spans="1:38" ht="32" x14ac:dyDescent="0.7">
-      <c r="B3" s="68" t="s">
+      <c r="B3" s="72" t="s">
         <v>511</v>
       </c>
-      <c r="C3" s="68"/>
-      <c r="D3" s="68"/>
-      <c r="E3" s="68"/>
-      <c r="F3" s="68"/>
-      <c r="G3" s="68"/>
-      <c r="H3" s="68"/>
-      <c r="I3" s="68"/>
-      <c r="J3" s="68"/>
-      <c r="K3" s="68"/>
-      <c r="L3" s="68"/>
-      <c r="M3" s="68"/>
-      <c r="N3" s="68"/>
-      <c r="O3" s="68"/>
-      <c r="P3" s="68"/>
-      <c r="Q3" s="68"/>
-      <c r="R3" s="68"/>
-      <c r="S3" s="68"/>
-      <c r="T3" s="68"/>
-      <c r="U3" s="68"/>
-      <c r="V3" s="68"/>
-      <c r="W3" s="68"/>
-      <c r="X3" s="68"/>
-      <c r="Y3" s="68"/>
-      <c r="Z3" s="68"/>
-      <c r="AA3" s="68"/>
-      <c r="AB3" s="68"/>
-      <c r="AC3" s="68"/>
-      <c r="AD3" s="68"/>
-      <c r="AE3" s="68"/>
-      <c r="AF3" s="68"/>
-      <c r="AG3" s="68"/>
-      <c r="AH3" s="68"/>
-      <c r="AI3" s="68"/>
-      <c r="AJ3" s="68"/>
+      <c r="C3" s="72"/>
+      <c r="D3" s="72"/>
+      <c r="E3" s="72"/>
+      <c r="F3" s="72"/>
+      <c r="G3" s="72"/>
+      <c r="H3" s="72"/>
+      <c r="I3" s="72"/>
+      <c r="J3" s="72"/>
+      <c r="K3" s="72"/>
+      <c r="L3" s="72"/>
+      <c r="M3" s="72"/>
+      <c r="N3" s="72"/>
+      <c r="O3" s="72"/>
+      <c r="P3" s="72"/>
+      <c r="Q3" s="72"/>
+      <c r="R3" s="72"/>
+      <c r="S3" s="72"/>
+      <c r="T3" s="72"/>
+      <c r="U3" s="72"/>
+      <c r="V3" s="72"/>
+      <c r="W3" s="72"/>
+      <c r="X3" s="72"/>
+      <c r="Y3" s="72"/>
+      <c r="Z3" s="72"/>
+      <c r="AA3" s="72"/>
+      <c r="AB3" s="72"/>
+      <c r="AC3" s="72"/>
+      <c r="AD3" s="72"/>
+      <c r="AE3" s="72"/>
+      <c r="AF3" s="72"/>
+      <c r="AG3" s="72"/>
+      <c r="AH3" s="72"/>
+      <c r="AI3" s="72"/>
+      <c r="AJ3" s="72"/>
     </row>
     <row r="4" spans="1:38" ht="29.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="19" t="s">
@@ -18864,18 +18856,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:8" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="B1" s="57" t="s">
+      <c r="B1" s="61" t="s">
         <v>36</v>
       </c>
-      <c r="C1" s="56"/>
-      <c r="D1" s="56"/>
+      <c r="C1" s="60"/>
+      <c r="D1" s="60"/>
     </row>
     <row r="2" spans="2:8" ht="35" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="55" t="s">
+      <c r="B2" s="59" t="s">
         <v>404</v>
       </c>
-      <c r="C2" s="56"/>
-      <c r="D2" s="56"/>
+      <c r="C2" s="60"/>
+      <c r="D2" s="60"/>
     </row>
     <row r="4" spans="2:8" ht="45" x14ac:dyDescent="0.35">
       <c r="B4" s="35" t="s">
@@ -18887,13 +18879,13 @@
       <c r="D4" s="36" t="s">
         <v>37</v>
       </c>
-      <c r="F4" s="69" t="s">
+      <c r="F4" s="55" t="s">
         <v>528</v>
       </c>
-      <c r="G4" s="69" t="s">
+      <c r="G4" s="55" t="s">
         <v>529</v>
       </c>
-      <c r="H4" s="69" t="s">
+      <c r="H4" s="55" t="s">
         <v>530</v>
       </c>
     </row>
@@ -18907,13 +18899,13 @@
       <c r="D5" s="37">
         <v>46203</v>
       </c>
-      <c r="F5" s="70" t="s">
+      <c r="F5" s="56" t="s">
         <v>531</v>
       </c>
-      <c r="G5" s="71">
+      <c r="G5" s="57">
         <v>165.92526540126542</v>
       </c>
-      <c r="H5" s="72">
+      <c r="H5" s="58">
         <v>135</v>
       </c>
     </row>
@@ -18927,13 +18919,13 @@
       <c r="D6" s="37">
         <v>46203</v>
       </c>
-      <c r="F6" s="70" t="s">
+      <c r="F6" s="56" t="s">
         <v>532</v>
       </c>
-      <c r="G6" s="71">
+      <c r="G6" s="57">
         <v>241.03174325966435</v>
       </c>
-      <c r="H6" s="72">
+      <c r="H6" s="58">
         <v>135</v>
       </c>
     </row>

</xml_diff>